<commit_message>
Clarify cohort demographics and supplementary labels and improve figure readability
</commit_message>
<xml_diff>
--- a/results/tables/Main_Tables.xlsx
+++ b/results/tables/Main_Tables.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -465,130 +465,174 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Eligible sequencing profiles</t>
+          <t>Sex, children, n (%)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>Female 12 (46.2%); Male 14 (53.8%)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>143</t>
+          <t>Female 10 (52.6%); Male 9 (47.4%)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>56; one adenoid and one tonsil per child</t>
+          <t>Not available in released input table</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Profiles per child, median (range)</t>
+          <t>Eligible sequencing profiles</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>5.5 (1–21)</t>
+          <t>180</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>7 (3–13)</t>
+          <t>143</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2 (2–2)</t>
+          <t>56; one adenoid and one tonsil per child</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Released initial age / observed age</t>
+          <t>Profiles per child, median (range)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Initial integer field 4–6 years</t>
+          <t>5.5 (1–21)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Initial integer field 4–6 years</t>
+          <t>7 (3–13)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Observed age 15–65 months (source Table 1)</t>
+          <t>2 (2–2)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Baseline daycare, children</t>
+          <t>Initial age, median (IQR), years</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>20/26</t>
+          <t>5 (4–5)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>16/19</t>
+          <t>5 (4–5)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Not used in anatomical analyses</t>
+          <t>Not available in released input table</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Household tobacco exposure, children</t>
+          <t>Released initial age / observed age</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>1/26</t>
+          <t>Initial integer field 4–6 years</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>0/19</t>
+          <t>Initial integer field 4–6 years</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Not used in anatomical analyses</t>
+          <t>Observed age 15–65 months (source Table 1)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>Baseline daycare, children</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>20/26</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>16/19</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Not used in anatomical analyses</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Household tobacco exposure, children</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>1/26</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>0/19</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Not used in anatomical analyses</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
           <t>Moraxella-dominant profile fraction per child, median</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>0.455</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>0.571</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t>Described by tissue</t>
         </is>

</xml_diff>